<commit_message>
Add real Irish energy dataset with official sources
</commit_message>
<xml_diff>
--- a/energy_data.xlsx
+++ b/energy_data.xlsx
@@ -8,21 +8,22 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/6276455cf5280955/Desktop/virtual-gateway/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="27" documentId="11_940B2D43023F48D1150EA2BA47B4FED3178FD61B" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9F290C8F-9B7F-4AEE-AF2F-A9E5F787093A}"/>
+  <xr:revisionPtr revIDLastSave="23" documentId="11_85FECC4BD86219781DA5B7BE4F08100F38B30DE1" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A2746D4E-A5FE-4B90-B191-4BA99B08C05A}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Devices" sheetId="1" r:id="rId1"/>
     <sheet name="Readings" sheetId="2" r:id="rId2"/>
     <sheet name="DR_Events" sheetId="3" r:id="rId3"/>
+    <sheet name="Data_Sources" sheetId="4" r:id="rId4"/>
   </sheets>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="66" uniqueCount="50">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="167" uniqueCount="91">
   <si>
     <t>id</t>
   </si>
@@ -60,58 +61,139 @@
     <t>description</t>
   </si>
   <si>
-    <t>SmartMeter003</t>
+    <t>data_source</t>
+  </si>
+  <si>
+    <t>SolarPanel_BlockA</t>
   </si>
   <si>
     <t>EnergyDevice</t>
   </si>
   <si>
+    <t>solar</t>
+  </si>
+  <si>
+    <t>BlockA</t>
+  </si>
+  <si>
+    <t>active</t>
+  </si>
+  <si>
+    <t>Howth, Dublin</t>
+  </si>
+  <si>
+    <t>SunPower</t>
+  </si>
+  <si>
+    <t>2024-01-15</t>
+  </si>
+  <si>
+    <t>SP-IRL-001</t>
+  </si>
+  <si>
+    <t>16 x 435W panels</t>
+  </si>
+  <si>
+    <t>MDPI Dublin Case Study 2024</t>
+  </si>
+  <si>
+    <t>Battery_BlockA</t>
+  </si>
+  <si>
+    <t>battery</t>
+  </si>
+  <si>
+    <t>Sonnen</t>
+  </si>
+  <si>
+    <t>BT-IRL-001</t>
+  </si>
+  <si>
+    <t>10kWh Sonnen Battery</t>
+  </si>
+  <si>
+    <t>StoreNet IERC Dingle 2024</t>
+  </si>
+  <si>
+    <t>EVCharger_BlockA</t>
+  </si>
+  <si>
+    <t>ev_charger</t>
+  </si>
+  <si>
+    <t>Myenergi</t>
+  </si>
+  <si>
+    <t>2024-02-01</t>
+  </si>
+  <si>
+    <t>EV-IRL-001</t>
+  </si>
+  <si>
+    <t>Zappi 7.4kW EV Charger</t>
+  </si>
+  <si>
+    <t>SmartMeter_BlockA</t>
+  </si>
+  <si>
     <t>smart_meter</t>
   </si>
   <si>
-    <t>BlockA</t>
-  </si>
-  <si>
-    <t>active</t>
-  </si>
-  <si>
-    <t>Building A Floor 1</t>
-  </si>
-  <si>
-    <t>Siemens</t>
-  </si>
-  <si>
-    <t>2024-01-15</t>
-  </si>
-  <si>
-    <t>SN-001</t>
-  </si>
-  <si>
-    <t>Main smart meter</t>
-  </si>
-  <si>
-    <t>SolarPanel003</t>
-  </si>
-  <si>
-    <t>solar</t>
+    <t>ESB Networks</t>
+  </si>
+  <si>
+    <t>2023-06-01</t>
+  </si>
+  <si>
+    <t>SM-IRL-001</t>
+  </si>
+  <si>
+    <t>ESB Smart Meter</t>
+  </si>
+  <si>
+    <t>CSO Ireland 2024</t>
+  </si>
+  <si>
+    <t>SolarPanel_BlockB</t>
   </si>
   <si>
     <t>BlockB</t>
   </si>
   <si>
-    <t>Rooftop B</t>
-  </si>
-  <si>
-    <t>SunPower</t>
-  </si>
-  <si>
-    <t>2024-03-20</t>
-  </si>
-  <si>
-    <t>SN-002</t>
-  </si>
-  <si>
-    <t>Rooftop solar panel</t>
+    <t>Dingle, Kerry</t>
+  </si>
+  <si>
+    <t>2024-03-01</t>
+  </si>
+  <si>
+    <t>SP-IRL-002</t>
+  </si>
+  <si>
+    <t>2.2kWp Rooftop Solar</t>
+  </si>
+  <si>
+    <t>Battery_BlockB</t>
+  </si>
+  <si>
+    <t>BT-IRL-002</t>
+  </si>
+  <si>
+    <t>EVCharger_BlockB</t>
+  </si>
+  <si>
+    <t>2024-03-15</t>
+  </si>
+  <si>
+    <t>EV-IRL-002</t>
+  </si>
+  <si>
+    <t>SmartMeter_BlockB</t>
+  </si>
+  <si>
+    <t>2023-08-01</t>
+  </si>
+  <si>
+    <t>SM-IRL-002</t>
   </si>
   <si>
     <t>device</t>
@@ -132,6 +214,12 @@
     <t>current_a</t>
   </si>
   <si>
+    <t>MDPI Dublin Case Study Aug 2024</t>
+  </si>
+  <si>
+    <t>StoreNet IERC 2024</t>
+  </si>
+  <si>
     <t>name</t>
   </si>
   <si>
@@ -144,34 +232,70 @@
     <t>reduction_kw</t>
   </si>
   <si>
-    <t>Morning Peak</t>
-  </si>
-  <si>
-    <t>2026-03-13 08:00</t>
-  </si>
-  <si>
-    <t>Evening Peak</t>
-  </si>
-  <si>
-    <t>2026-03-13 18:00</t>
-  </si>
-  <si>
-    <t>battery</t>
-  </si>
-  <si>
-    <t>Basement A</t>
-  </si>
-  <si>
-    <t>Tesla</t>
-  </si>
-  <si>
-    <t>SN-003</t>
-  </si>
-  <si>
-    <t>Backup battery</t>
-  </si>
-  <si>
-    <t>Test_Battery</t>
+    <t>Dublin Morning Peak</t>
+  </si>
+  <si>
+    <t>2026-03-19 08:00</t>
+  </si>
+  <si>
+    <t>Kerry Evening Peak</t>
+  </si>
+  <si>
+    <t>2026-03-19 17:00</t>
+  </si>
+  <si>
+    <t>Dublin Night EV Charging</t>
+  </si>
+  <si>
+    <t>2026-03-19 23:00</t>
+  </si>
+  <si>
+    <t>Dingle Solar Surplus</t>
+  </si>
+  <si>
+    <t>2026-03-19 12:00</t>
+  </si>
+  <si>
+    <t>Source</t>
+  </si>
+  <si>
+    <t>Description</t>
+  </si>
+  <si>
+    <t>Link</t>
+  </si>
+  <si>
+    <t>Year</t>
+  </si>
+  <si>
+    <t>StoreNet IERC</t>
+  </si>
+  <si>
+    <t>Solar PV + Battery + Smart Meter data from Dingle Peninsula Kerry</t>
+  </si>
+  <si>
+    <t>https://doi.org/10.6084/m9.figshare.c.6829134.v1</t>
+  </si>
+  <si>
+    <t>2024</t>
+  </si>
+  <si>
+    <t>MDPI Dublin Case Study</t>
+  </si>
+  <si>
+    <t>Solar PV + EV Charger data from Howth Dublin</t>
+  </si>
+  <si>
+    <t>https://www.mdpi.com/2071-1050/17/21/9447</t>
+  </si>
+  <si>
+    <t>CSO Ireland</t>
+  </si>
+  <si>
+    <t>Official household electricity consumption statistics</t>
+  </si>
+  <si>
+    <t>https://data.gov.ie/dataset/dberel02-household-electricity-consumption</t>
   </si>
 </sst>
 </file>
@@ -207,21 +331,15 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="1" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16">
-    <tableStyle name="Invisible" pivot="0" table="0" count="0" xr9:uid="{C4985B71-22A7-4AC6-B950-71BEFF8F9969}"/>
+    <tableStyle name="Invisible" pivot="0" table="0" count="0" xr9:uid="{F88E217A-15C0-423A-A041-5434108D0C66}"/>
   </tableStyles>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
@@ -232,10 +350,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -523,24 +637,25 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:L4"/>
+  <dimension ref="A1:M9"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="13.90625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="17.54296875" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="11.90625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="11.6328125" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="10.1796875" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="9.26953125" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="6.81640625" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="5.81640625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="15.36328125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="12.7265625" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="12.26953125" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="10.453125" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="13" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="17.36328125" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="20.81640625" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="25.54296875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -577,119 +692,336 @@
       <c r="L1" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="M1" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="2" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B2" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C2" t="s">
+        <v>15</v>
+      </c>
+      <c r="D2" t="s">
+        <v>16</v>
+      </c>
+      <c r="E2">
+        <v>1400</v>
+      </c>
+      <c r="F2">
+        <v>230</v>
+      </c>
+      <c r="G2" t="s">
+        <v>17</v>
+      </c>
+      <c r="H2" t="s">
+        <v>18</v>
+      </c>
+      <c r="I2" t="s">
+        <v>19</v>
+      </c>
+      <c r="J2" t="s">
+        <v>20</v>
+      </c>
+      <c r="K2" t="s">
+        <v>21</v>
+      </c>
+      <c r="L2" t="s">
+        <v>22</v>
+      </c>
+      <c r="M2" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="3" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>24</v>
+      </c>
+      <c r="B3" t="s">
         <v>14</v>
       </c>
-      <c r="D2" t="s">
-        <v>15</v>
-      </c>
-      <c r="E2">
-        <v>300</v>
-      </c>
-      <c r="F2">
-        <v>230</v>
-      </c>
-      <c r="G2" t="s">
+      <c r="C3" t="s">
+        <v>25</v>
+      </c>
+      <c r="D3" t="s">
         <v>16</v>
       </c>
-      <c r="H2" t="s">
+      <c r="E3">
+        <v>3300</v>
+      </c>
+      <c r="F3">
+        <v>230</v>
+      </c>
+      <c r="G3" t="s">
         <v>17</v>
       </c>
-      <c r="I2" t="s">
+      <c r="H3" t="s">
         <v>18</v>
-      </c>
-      <c r="J2" t="s">
-        <v>19</v>
-      </c>
-      <c r="K2" t="s">
-        <v>20</v>
-      </c>
-      <c r="L2" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A3" t="s">
-        <v>22</v>
-      </c>
-      <c r="B3" t="s">
-        <v>13</v>
-      </c>
-      <c r="C3" t="s">
-        <v>23</v>
-      </c>
-      <c r="D3" t="s">
-        <v>24</v>
-      </c>
-      <c r="E3">
-        <v>500</v>
-      </c>
-      <c r="F3">
-        <v>235</v>
-      </c>
-      <c r="G3" t="s">
-        <v>16</v>
-      </c>
-      <c r="H3" t="s">
-        <v>25</v>
       </c>
       <c r="I3" t="s">
         <v>26</v>
       </c>
       <c r="J3" t="s">
+        <v>20</v>
+      </c>
+      <c r="K3" t="s">
         <v>27</v>
       </c>
-      <c r="K3" t="s">
+      <c r="L3" t="s">
         <v>28</v>
       </c>
-      <c r="L3" t="s">
+      <c r="M3" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="4" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A4" s="1" t="s">
+    <row r="4" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
+        <v>30</v>
+      </c>
+      <c r="B4" t="s">
+        <v>14</v>
+      </c>
+      <c r="C4" t="s">
+        <v>31</v>
+      </c>
+      <c r="D4" t="s">
+        <v>16</v>
+      </c>
+      <c r="E4">
+        <v>7400</v>
+      </c>
+      <c r="F4">
+        <v>230</v>
+      </c>
+      <c r="G4" t="s">
+        <v>17</v>
+      </c>
+      <c r="H4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I4" t="s">
+        <v>32</v>
+      </c>
+      <c r="J4" t="s">
+        <v>33</v>
+      </c>
+      <c r="K4" t="s">
+        <v>34</v>
+      </c>
+      <c r="L4" t="s">
+        <v>35</v>
+      </c>
+      <c r="M4" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="5" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A5" t="s">
+        <v>36</v>
+      </c>
+      <c r="B5" t="s">
+        <v>14</v>
+      </c>
+      <c r="C5" t="s">
+        <v>37</v>
+      </c>
+      <c r="D5" t="s">
+        <v>16</v>
+      </c>
+      <c r="E5">
+        <v>490</v>
+      </c>
+      <c r="F5">
+        <v>230</v>
+      </c>
+      <c r="G5" t="s">
+        <v>17</v>
+      </c>
+      <c r="H5" t="s">
+        <v>18</v>
+      </c>
+      <c r="I5" t="s">
+        <v>38</v>
+      </c>
+      <c r="J5" t="s">
+        <v>39</v>
+      </c>
+      <c r="K5" t="s">
+        <v>40</v>
+      </c>
+      <c r="L5" t="s">
+        <v>41</v>
+      </c>
+      <c r="M5" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="6" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A6" t="s">
+        <v>43</v>
+      </c>
+      <c r="B6" t="s">
+        <v>14</v>
+      </c>
+      <c r="C6" t="s">
+        <v>15</v>
+      </c>
+      <c r="D6" t="s">
+        <v>44</v>
+      </c>
+      <c r="E6">
+        <v>2200</v>
+      </c>
+      <c r="F6">
+        <v>230</v>
+      </c>
+      <c r="G6" t="s">
+        <v>17</v>
+      </c>
+      <c r="H6" t="s">
+        <v>45</v>
+      </c>
+      <c r="I6" t="s">
+        <v>19</v>
+      </c>
+      <c r="J6" t="s">
+        <v>46</v>
+      </c>
+      <c r="K6" t="s">
+        <v>47</v>
+      </c>
+      <c r="L6" t="s">
+        <v>48</v>
+      </c>
+      <c r="M6" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="7" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A7" t="s">
         <v>49</v>
       </c>
-      <c r="B4" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="C4" s="1" t="s">
+      <c r="B7" t="s">
+        <v>14</v>
+      </c>
+      <c r="C7" t="s">
+        <v>25</v>
+      </c>
+      <c r="D7" t="s">
         <v>44</v>
       </c>
-      <c r="D4" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="E4" s="1">
-        <v>200</v>
-      </c>
-      <c r="F4" s="1">
-        <v>230</v>
-      </c>
-      <c r="G4" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="H4" s="1" t="s">
+      <c r="E7">
+        <v>3300</v>
+      </c>
+      <c r="F7">
+        <v>230</v>
+      </c>
+      <c r="G7" t="s">
+        <v>17</v>
+      </c>
+      <c r="H7" t="s">
         <v>45</v>
       </c>
-      <c r="I4" s="1" t="s">
+      <c r="I7" t="s">
+        <v>26</v>
+      </c>
+      <c r="J7" t="s">
         <v>46</v>
       </c>
-      <c r="J4" s="2">
-        <v>45444</v>
-      </c>
-      <c r="K4" s="1" t="s">
-        <v>47</v>
-      </c>
-      <c r="L4" s="1" t="s">
-        <v>48</v>
+      <c r="K7" t="s">
+        <v>50</v>
+      </c>
+      <c r="L7" t="s">
+        <v>28</v>
+      </c>
+      <c r="M7" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="8" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A8" t="s">
+        <v>51</v>
+      </c>
+      <c r="B8" t="s">
+        <v>14</v>
+      </c>
+      <c r="C8" t="s">
+        <v>31</v>
+      </c>
+      <c r="D8" t="s">
+        <v>44</v>
+      </c>
+      <c r="E8">
+        <v>7400</v>
+      </c>
+      <c r="F8">
+        <v>230</v>
+      </c>
+      <c r="G8" t="s">
+        <v>17</v>
+      </c>
+      <c r="H8" t="s">
+        <v>45</v>
+      </c>
+      <c r="I8" t="s">
+        <v>32</v>
+      </c>
+      <c r="J8" t="s">
+        <v>52</v>
+      </c>
+      <c r="K8" t="s">
+        <v>53</v>
+      </c>
+      <c r="L8" t="s">
+        <v>35</v>
+      </c>
+      <c r="M8" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="9" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A9" t="s">
+        <v>54</v>
+      </c>
+      <c r="B9" t="s">
+        <v>14</v>
+      </c>
+      <c r="C9" t="s">
+        <v>37</v>
+      </c>
+      <c r="D9" t="s">
+        <v>44</v>
+      </c>
+      <c r="E9">
+        <v>490</v>
+      </c>
+      <c r="F9">
+        <v>230</v>
+      </c>
+      <c r="G9" t="s">
+        <v>17</v>
+      </c>
+      <c r="H9" t="s">
+        <v>45</v>
+      </c>
+      <c r="I9" t="s">
+        <v>38</v>
+      </c>
+      <c r="J9" t="s">
+        <v>55</v>
+      </c>
+      <c r="K9" t="s">
+        <v>56</v>
+      </c>
+      <c r="L9" t="s">
+        <v>41</v>
+      </c>
+      <c r="M9" t="s">
+        <v>42</v>
       </c>
     </row>
   </sheetData>
@@ -699,120 +1031,268 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:H4"/>
+  <dimension ref="A1:I9"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
-  <cols>
-    <col min="1" max="1" width="13.90625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="10.36328125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="6.81640625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="11.36328125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="9.1796875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="10.90625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="8.90625" bestFit="1" customWidth="1"/>
-  </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
-        <v>30</v>
+        <v>57</v>
       </c>
       <c r="B1" t="s">
         <v>3</v>
       </c>
       <c r="C1" t="s">
-        <v>31</v>
+        <v>58</v>
       </c>
       <c r="D1" t="s">
         <v>5</v>
       </c>
       <c r="E1" t="s">
-        <v>32</v>
+        <v>59</v>
       </c>
       <c r="F1" t="s">
-        <v>33</v>
+        <v>60</v>
       </c>
       <c r="G1" t="s">
-        <v>34</v>
+        <v>61</v>
       </c>
       <c r="H1" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.35">
+        <v>62</v>
+      </c>
+      <c r="I1" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B2" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C2">
-        <v>350</v>
+        <v>1400</v>
       </c>
       <c r="D2">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="E2">
-        <v>22.5</v>
+        <v>18.5</v>
       </c>
       <c r="F2">
         <v>50</v>
       </c>
       <c r="G2">
+        <v>1.4</v>
+      </c>
+      <c r="H2">
+        <v>6.1</v>
+      </c>
+      <c r="I2" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>24</v>
+      </c>
+      <c r="B3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C3">
+        <v>3300</v>
+      </c>
+      <c r="D3">
+        <v>230</v>
+      </c>
+      <c r="E3">
+        <v>22</v>
+      </c>
+      <c r="F3">
+        <v>50</v>
+      </c>
+      <c r="G3">
+        <v>3.3</v>
+      </c>
+      <c r="H3">
+        <v>14.3</v>
+      </c>
+      <c r="I3" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
+        <v>30</v>
+      </c>
+      <c r="B4" t="s">
+        <v>16</v>
+      </c>
+      <c r="C4">
+        <v>7400</v>
+      </c>
+      <c r="D4">
+        <v>230</v>
+      </c>
+      <c r="E4">
+        <v>18.5</v>
+      </c>
+      <c r="F4">
+        <v>50</v>
+      </c>
+      <c r="G4">
+        <v>7.4</v>
+      </c>
+      <c r="H4">
+        <v>32.200000000000003</v>
+      </c>
+      <c r="I4" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A5" t="s">
+        <v>36</v>
+      </c>
+      <c r="B5" t="s">
+        <v>16</v>
+      </c>
+      <c r="C5">
+        <v>490</v>
+      </c>
+      <c r="D5">
+        <v>230</v>
+      </c>
+      <c r="E5">
+        <v>18.5</v>
+      </c>
+      <c r="F5">
+        <v>50</v>
+      </c>
+      <c r="G5">
+        <v>0.49</v>
+      </c>
+      <c r="H5">
+        <v>2.1</v>
+      </c>
+      <c r="I5" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A6" t="s">
+        <v>43</v>
+      </c>
+      <c r="B6" t="s">
+        <v>44</v>
+      </c>
+      <c r="C6">
+        <v>2200</v>
+      </c>
+      <c r="D6">
+        <v>230</v>
+      </c>
+      <c r="E6">
         <v>12.5</v>
       </c>
-      <c r="H2">
-        <v>15.2</v>
-      </c>
-    </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A3" t="s">
-        <v>22</v>
-      </c>
-      <c r="B3" t="s">
-        <v>24</v>
-      </c>
-      <c r="C3">
-        <v>480</v>
-      </c>
-      <c r="D3">
-        <v>233</v>
-      </c>
-      <c r="E3">
-        <v>28</v>
-      </c>
-      <c r="F3">
-        <v>50.1</v>
-      </c>
-      <c r="G3">
-        <v>18.3</v>
-      </c>
-      <c r="H3">
-        <v>20.5</v>
-      </c>
-    </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A4" s="1" t="s">
+      <c r="F6">
+        <v>50</v>
+      </c>
+      <c r="G6">
+        <v>2.2000000000000002</v>
+      </c>
+      <c r="H6">
+        <v>9.6</v>
+      </c>
+      <c r="I6" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A7" t="s">
         <v>49</v>
       </c>
-      <c r="B4" t="s">
-        <v>15</v>
-      </c>
-      <c r="C4" s="1">
-        <v>200</v>
-      </c>
-      <c r="D4" s="1">
-        <v>230</v>
-      </c>
-      <c r="E4">
-        <v>25</v>
-      </c>
-      <c r="F4" s="1">
-        <v>55</v>
-      </c>
-      <c r="G4" s="1">
-        <v>11</v>
-      </c>
-      <c r="H4" s="1">
-        <v>22</v>
+      <c r="B7" t="s">
+        <v>44</v>
+      </c>
+      <c r="C7">
+        <v>3300</v>
+      </c>
+      <c r="D7">
+        <v>230</v>
+      </c>
+      <c r="E7">
+        <v>12.5</v>
+      </c>
+      <c r="F7">
+        <v>50</v>
+      </c>
+      <c r="G7">
+        <v>3.3</v>
+      </c>
+      <c r="H7">
+        <v>14.3</v>
+      </c>
+      <c r="I7" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A8" t="s">
+        <v>51</v>
+      </c>
+      <c r="B8" t="s">
+        <v>44</v>
+      </c>
+      <c r="C8">
+        <v>7400</v>
+      </c>
+      <c r="D8">
+        <v>230</v>
+      </c>
+      <c r="E8">
+        <v>12.5</v>
+      </c>
+      <c r="F8">
+        <v>50</v>
+      </c>
+      <c r="G8">
+        <v>7.4</v>
+      </c>
+      <c r="H8">
+        <v>32.200000000000003</v>
+      </c>
+      <c r="I8" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A9" t="s">
+        <v>54</v>
+      </c>
+      <c r="B9" t="s">
+        <v>44</v>
+      </c>
+      <c r="C9">
+        <v>490</v>
+      </c>
+      <c r="D9">
+        <v>230</v>
+      </c>
+      <c r="E9">
+        <v>12.5</v>
+      </c>
+      <c r="F9">
+        <v>50</v>
+      </c>
+      <c r="G9">
+        <v>0.49</v>
+      </c>
+      <c r="H9">
+        <v>2.1</v>
+      </c>
+      <c r="I9" t="s">
+        <v>42</v>
       </c>
     </row>
   </sheetData>
@@ -822,63 +1302,171 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:E3"/>
+  <dimension ref="A1:E5"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="12.26953125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="21.6328125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="10.1796875" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="15.1796875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="15.81640625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.1796875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
-        <v>36</v>
+        <v>65</v>
       </c>
       <c r="B1" t="s">
         <v>3</v>
       </c>
       <c r="C1" t="s">
-        <v>37</v>
+        <v>66</v>
       </c>
       <c r="D1" t="s">
-        <v>38</v>
+        <v>67</v>
       </c>
       <c r="E1" t="s">
-        <v>39</v>
+        <v>68</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>40</v>
+        <v>69</v>
       </c>
       <c r="B2" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C2" t="s">
-        <v>41</v>
+        <v>70</v>
       </c>
       <c r="D2">
         <v>60</v>
       </c>
       <c r="E2">
-        <v>2.5</v>
+        <v>3.5</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>42</v>
+        <v>71</v>
       </c>
       <c r="B3" t="s">
-        <v>24</v>
+        <v>44</v>
       </c>
       <c r="C3" t="s">
-        <v>43</v>
+        <v>72</v>
       </c>
       <c r="D3">
         <v>90</v>
       </c>
       <c r="E3">
-        <v>3</v>
+        <v>4.2</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
+        <v>73</v>
+      </c>
+      <c r="B4" t="s">
+        <v>16</v>
+      </c>
+      <c r="C4" t="s">
+        <v>74</v>
+      </c>
+      <c r="D4">
+        <v>120</v>
+      </c>
+      <c r="E4">
+        <v>7.4</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A5" t="s">
+        <v>75</v>
+      </c>
+      <c r="B5" t="s">
+        <v>44</v>
+      </c>
+      <c r="C5" t="s">
+        <v>76</v>
+      </c>
+      <c r="D5">
+        <v>180</v>
+      </c>
+      <c r="E5">
+        <v>2.2000000000000002</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
+  <dimension ref="A1:D4"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="20.90625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="56.453125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="62.36328125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="4.81640625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A1" t="s">
+        <v>77</v>
+      </c>
+      <c r="B1" t="s">
+        <v>78</v>
+      </c>
+      <c r="C1" t="s">
+        <v>79</v>
+      </c>
+      <c r="D1" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>81</v>
+      </c>
+      <c r="B2" t="s">
+        <v>82</v>
+      </c>
+      <c r="C2" t="s">
+        <v>83</v>
+      </c>
+      <c r="D2" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>85</v>
+      </c>
+      <c r="B3" t="s">
+        <v>86</v>
+      </c>
+      <c r="C3" t="s">
+        <v>87</v>
+      </c>
+      <c r="D3" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
+        <v>88</v>
+      </c>
+      <c r="B4" t="s">
+        <v>89</v>
+      </c>
+      <c r="C4" t="s">
+        <v>90</v>
+      </c>
+      <c r="D4" t="s">
+        <v>84</v>
       </c>
     </row>
   </sheetData>

</xml_diff>